<commit_message>
SOIL_parameters workbooks: a note on every column
Adds notes for Soil_type, Index, the three Ks multipliers, Ltop_m, dh_max_m and l_vg, and
states how the layered subsurface treats Sy (ignored), kgsat (rock Kh fallback) and DTB
(not read by the current code). Cell values and the logo image are unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Examples/Stanford/Input_Data_Sheets/SOIL_parameters.xlsx
+++ b/Examples/Stanford/Input_Data_Sheets/SOIL_parameters.xlsx
@@ -423,58 +423,106 @@
     <author>Marcus Gomes</author>
   </authors>
   <commentList>
+    <comment ref="A2" authorId="0" shapeId="0">
+      <text>
+        <t xml:space="preserve">Marcus Gomes:
+Soil class name, for your reference only.</t>
+      </text>
+    </comment>
+    <comment ref="B2" authorId="0" shapeId="0">
+      <text>
+        <t xml:space="preserve">Marcus Gomes:
+Soil class code. It must match the cell values of the SOIL raster (SOIL_path in General_Data). One row per class.</t>
+      </text>
+    </comment>
     <comment ref="C2" authorId="0" shapeId="0">
       <text>
         <t xml:space="preserve">Marcus Gomes:
-Saturated Hydraulic Conductivity </t>
+Saturated hydraulic conductivity of the soil, in mm/h. Used for infiltration and for drainage through the three soil layers; the three Ks multipliers scale it per layer.</t>
       </text>
     </comment>
     <comment ref="D2" authorId="0" shapeId="0">
       <text>
-        <t>Marcus Gomes:
-van-Genutchen n parameter</t>
+        <t xml:space="preserve">Marcus Gomes:
+van Genuchten n of the soil (dimensionless, greater than 1).</t>
       </text>
     </comment>
     <comment ref="E2" authorId="0" shapeId="0">
       <text>
-        <t>Marcus Gomes:
-van-Genutchen alpha parameter</t>
+        <t xml:space="preserve">Marcus Gomes:
+van Genuchten alpha of the soil, in 1/m.</t>
       </text>
     </comment>
     <comment ref="F2" authorId="0" shapeId="0">
       <text>
-        <t>Marcus Gomes:
-Saturated porosity</t>
+        <t xml:space="preserve">Marcus Gomes:
+Saturated water content (porosity) of the soil, cm3/cm3.</t>
       </text>
     </comment>
     <comment ref="G2" authorId="0" shapeId="0">
       <text>
-        <t>Marcus Gomes:
-Residual porosity</t>
+        <t xml:space="preserve">Marcus Gomes:
+Residual water content of the soil, cm3/cm3.</t>
       </text>
     </comment>
     <comment ref="H2" authorId="0" shapeId="0">
       <text>
-        <t>Marcus Gomes:
-Initial water content</t>
+        <t xml:space="preserve">Marcus Gomes:
+Initial water content of the soil layers at the start of the run, cm3/cm3, between the residual and saturated values.</t>
       </text>
     </comment>
     <comment ref="I2" authorId="0" shapeId="0">
       <text>
-        <t>Marcus Gomes:
-Shallow aquifer drainable porosity</t>
+        <t xml:space="preserve">Marcus Gomes:
+Specific yield (drainable porosity) of the shallow aquifer. Legacy groundwater only. The layered subsurface ignores this column: Sy comes from each layer's van Genuchten curve (theta_sat minus the water content at field capacity).</t>
       </text>
     </comment>
     <comment ref="J2" authorId="0" shapeId="0">
       <text>
-        <t>Marcus Gomes:
-Lateral saturated hydraulic conductivity for shallow aquifer</t>
+        <t xml:space="preserve">Marcus Gomes:
+Lateral saturated hydraulic conductivity of the shallow aquifer, in mm/h. Legacy groundwater: the aquifer conductivity. Layered subsurface: the horizontal conductivity of the rock layers when regolith_ksat_h_mm_h and RegolithKsatH_path (General_Data) are empty.</t>
       </text>
     </comment>
     <comment ref="K2" authorId="0" shapeId="0">
       <text>
-        <t>Marcus Gomes:
-Distance to bedrock</t>
+        <t xml:space="preserve">Marcus Gomes:
+Depth to bedrock per soil class, in metres. Not read by the current MATLAB code: the soil depth comes from DTB_path, or 1 m when DTB_path is empty.</t>
+      </text>
+    </comment>
+    <comment ref="L2" authorId="0" shapeId="0">
+      <text>
+        <t xml:space="preserve">Marcus Gomes:
+Multiplier of ksat in the near-surface soil layer (thickness Ltop_m). Use less than 1 for crusted or compacted surfaces. 1 = no change.</t>
+      </text>
+    </comment>
+    <comment ref="M2" authorId="0" shapeId="0">
+      <text>
+        <t xml:space="preserve">Marcus Gomes:
+Multiplier of ksat in the root-zone soil layer (from Ltop_m down to the root depth of LULC_parameters.xlsx). 1 = no change.</t>
+      </text>
+    </comment>
+    <comment ref="N2" authorId="0" shapeId="0">
+      <text>
+        <t xml:space="preserve">Marcus Gomes:
+Multiplier of ksat in the transmission soil layer (from the root depth down to the bottom of the soil). 1 = no change.</t>
+      </text>
+    </comment>
+    <comment ref="O2" authorId="0" shapeId="0">
+      <text>
+        <t xml:space="preserve">Marcus Gomes:
+Thickness of the near-surface soil layer, in metres. It is also the length scale of the infiltration capacity: C = Ks x [min(h0 - h(theta), dh_max) / Ltop + 1].</t>
+      </text>
+    </comment>
+    <comment ref="P2" authorId="0" shapeId="0">
+      <text>
+        <t xml:space="preserve">Marcus Gomes:
+Cap on the driving head difference in the infiltration capacity, in metres: C = Ks x [min(h0 - h(theta), dh_max) / Ltop + 1]. Default 1 m.</t>
+      </text>
+    </comment>
+    <comment ref="Q2" authorId="0" shapeId="0">
+      <text>
+        <t xml:space="preserve">Marcus Gomes:
+Mualem pore-connectivity parameter l of the van Genuchten-Mualem unsaturated conductivity (dimensionless; 0.5 is the usual value).</t>
       </text>
     </comment>
   </commentList>

</xml_diff>